<commit_message>
docs: reconcile canon and project contracts
</commit_message>
<xml_diff>
--- a/source-documents/ОЧЕРЕДЬ_ИССЛЕДОВАНИЙ_СТРАН.xlsx
+++ b/source-documents/ОЧЕРЕДЬ_ИССЛЕДОВАНИЙ_СТРАН.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Очередь исследований" sheetId="1" r:id="Rb3c57e03147d49fc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Очередь исследований" sheetId="1" r:id="Rc005477d41654f9f"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -81,7 +81,7 @@
         <x:color rgb="FF17613B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFDDF3E5"/>
         </x:patternFill>
       </x:fill>
@@ -91,7 +91,7 @@
         <x:color rgb="FF174F9B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFEAF2FF"/>
         </x:patternFill>
       </x:fill>
@@ -102,7 +102,7 @@
         <x:color rgb="FF8B2638"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFDE9ED"/>
         </x:patternFill>
       </x:fill>
@@ -460,7 +460,7 @@
         <x:v>Признан однополый брак</x:v>
       </x:c>
       <x:c r="E8" s="9" t="str">
-        <x:v>В очереди</x:v>
+        <x:v>Подключена</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="22" customHeight="1">
@@ -477,7 +477,7 @@
         <x:v>Признан однополый брак</x:v>
       </x:c>
       <x:c r="E9" s="9" t="str">
-        <x:v>В очереди</x:v>
+        <x:v>Подключена</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="22" customHeight="1">
@@ -494,7 +494,7 @@
         <x:v>Признан однополый брак</x:v>
       </x:c>
       <x:c r="E10" s="9" t="str">
-        <x:v>В очереди</x:v>
+        <x:v>Подключена</x:v>
       </x:c>
     </x:row>
     <x:row r="11" ht="22" customHeight="1">
@@ -511,7 +511,7 @@
         <x:v>Признан однополый брак</x:v>
       </x:c>
       <x:c r="E11" s="9" t="str">
-        <x:v>В очереди</x:v>
+        <x:v>Подключена</x:v>
       </x:c>
     </x:row>
     <x:row r="12" ht="22" customHeight="1">
@@ -528,7 +528,7 @@
         <x:v>Признан однополый брак</x:v>
       </x:c>
       <x:c r="E12" s="9" t="str">
-        <x:v>В очереди</x:v>
+        <x:v>Подключена</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="22" customHeight="1">
@@ -545,7 +545,7 @@
         <x:v>Признан однополый брак</x:v>
       </x:c>
       <x:c r="E13" s="9" t="str">
-        <x:v>В очереди</x:v>
+        <x:v>Подключена</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="22" customHeight="1">
@@ -1650,7 +1650,7 @@
         <x:v>Частично признаны права пары</x:v>
       </x:c>
       <x:c r="E78" s="9" t="str">
-        <x:v>В очереди</x:v>
+        <x:v>Подключена</x:v>
       </x:c>
     </x:row>
     <x:row r="79" ht="22" customHeight="1">
@@ -4607,7 +4607,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rc3d2dd5a352f4c04"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re40636cfd09e42ca"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>

<commit_message>
feat: add Malta 15.0.0
</commit_message>
<xml_diff>
--- a/source-documents/ОЧЕРЕДЬ_ИССЛЕДОВАНИЙ_СТРАН.xlsx
+++ b/source-documents/ОЧЕРЕДЬ_ИССЛЕДОВАНИЙ_СТРАН.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Очередь исследований" sheetId="1" r:id="Rc005477d41654f9f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Очередь исследований" sheetId="1" r:id="R88499e95c6f24816"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -562,7 +562,7 @@
         <x:v>Признан однополый брак</x:v>
       </x:c>
       <x:c r="E14" s="9" t="str">
-        <x:v>В очереди</x:v>
+        <x:v>Подключена</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="22" customHeight="1">
@@ -4607,7 +4607,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Re40636cfd09e42ca"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R38f2a05840624d17"/>
   </x:tableParts>
 </x:worksheet>
 </file>
</xml_diff>